<commit_message>
docs: controlled vocabularies updated instructions
</commit_message>
<xml_diff>
--- a/Documents/Controlled_Vocabularies_Instructions.xlsx
+++ b/Documents/Controlled_Vocabularies_Instructions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthri.sharepoint.com/sites/hri-team022/Shared Documents/05 - FAIR/Workplan &amp; Activities/2025/D1_Metadata, data modeling and library/1.Metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{234C5A3E-8195-42B9-AE22-7AF9E95FEDB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{027CF694-BCEA-4479-A1BF-AC0FDE82ED29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C3D56D4C-58DE-344E-9B77-FB88BD7D2C37}"/>
   </bookViews>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="183">
   <si>
     <t>Class</t>
   </si>
@@ -101,7 +101,7 @@
     <t>http://publications.europa.eu/resource/authority/access-right</t>
   </si>
   <si>
-    <t xml:space="preserve">The EU authority table, containing values for access rights of the Dataset. You can choose between the values PUBLIC, NON_PUBLIC and RESTRICTED, even though in the vocabulary itself more values are included. Depending on the value that is choosed here, one of the three different versions of HealthCAT-AP will be used. </t>
+    <t xml:space="preserve">The EU authority table, containing values for access rights of the Dataset. You can choose between the values PUBLIC, NON_PUBLIC and RESTRICTED, even though in the vocabulary itself more values are included. Depending on the value that is choosed here, one of the three different versions of HealthDCAT-AP will be used. </t>
   </si>
   <si>
     <t>http://publications.europa.eu/resource/authority/access-right/PUBLIC</t>
@@ -290,7 +290,7 @@
     <t>http://publications.europa.eu/resource/authority/dataset-type</t>
   </si>
   <si>
-    <t>Choose the type of the dataset in the EU authority table. Choose the theme(s) of the dataset in the EU authority table.</t>
+    <t>Choose the type of the dataset in the EU authority table.</t>
   </si>
   <si>
     <t>http://publications.europa.eu/resource/authority/dataset-type/SYNTHETIC_DATA</t>
@@ -457,10 +457,97 @@
     <t>Choose the language of the distribution in the EU authority table.</t>
   </si>
   <si>
-    <t>Choose a license that is applicable to your distribution. You can choose one from the DCAT-AP NL provided list, which uses Creative Commons licenses. If you need help choosing one, it is recommended to use the chooser tool from Creative Commons (https://creativecommons.org/chooser/).</t>
-  </si>
-  <si>
-    <t>&lt;http://example.healthdata.nl/set/distribution&gt; dct:license &lt;https://creativecommons.org/licenses/by/4.0/&gt;.</t>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>For license of Distribution, please choose between "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>not-open" licence</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for non-public data or "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CC0"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for public data.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Non-public data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: https://definities.geostandaarden.nl/dcat-ap-nl/id/waardelijst/licenties/niet_open 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Public data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: http://creativecommons.org/publicdomain/zero/1.0/deed.nl</t>
+    </r>
+  </si>
+  <si>
+    <t>&lt;http://example.healthdata.nl/set/distribution&gt; dct:license &lt;https://creativecommons.org/publicdomain/zero/1.0/deed.nl&gt;.</t>
   </si>
   <si>
     <t>media type</t>
@@ -688,7 +775,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -744,6 +831,19 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -766,7 +866,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -794,6 +894,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1838,7 +1941,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="90.75">
+    <row r="22" spans="1:8" ht="88.5" customHeight="1">
       <c r="A22" s="5" t="s">
         <v>109</v>
       </c>
@@ -1851,14 +1954,14 @@
       <c r="D22" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>86</v>
+      <c r="F22" s="13" t="s">
+        <v>125</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H22" s="7"/>
     </row>
@@ -1867,22 +1970,22 @@
         <v>109</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>112</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H23" s="7"/>
     </row>
@@ -1891,22 +1994,22 @@
         <v>109</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>112</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H24" s="7"/>
     </row>
@@ -1921,24 +2024,24 @@
         <v>56</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="54.75">
       <c r="A26" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>16</v>
@@ -1950,13 +2053,13 @@
         <v>18</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H26" s="12" t="s">
         <v>22</v>
@@ -1964,7 +2067,7 @@
     </row>
     <row r="27" spans="1:8" ht="199.5">
       <c r="A27" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>23</v>
@@ -1976,21 +2079,21 @@
         <v>25</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="54.75">
       <c r="A28" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>9</v>
@@ -2002,13 +2105,13 @@
         <v>11</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H28" s="12" t="s">
         <v>15</v>
@@ -2016,7 +2119,7 @@
     </row>
     <row r="29" spans="1:8" ht="46.5">
       <c r="A29" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>116</v>
@@ -2028,13 +2131,13 @@
         <v>118</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H29" s="12" t="s">
         <v>122</v>
@@ -2042,7 +2145,7 @@
     </row>
     <row r="30" spans="1:8" ht="46.5">
       <c r="A30" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>30</v>
@@ -2054,13 +2157,13 @@
         <v>32</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>34</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H30" s="12" t="s">
         <v>36</v>
@@ -2068,7 +2171,7 @@
     </row>
     <row r="31" spans="1:8" ht="90.75">
       <c r="A31" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>82</v>
@@ -2080,19 +2183,19 @@
         <v>84</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>86</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H31" s="7"/>
     </row>
     <row r="32" spans="1:8" ht="46.5">
       <c r="A32" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>62</v>
@@ -2101,16 +2204,16 @@
         <v>63</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F32" s="7" t="s">
         <v>66</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H32" s="12" t="s">
         <v>68</v>
@@ -2118,73 +2221,73 @@
     </row>
     <row r="33" spans="1:8" ht="90.75">
       <c r="A33" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H33" s="7"/>
     </row>
     <row r="34" spans="1:8" ht="90.75">
       <c r="A34" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H34" s="7"/>
     </row>
     <row r="35" spans="1:8" ht="72.75">
       <c r="A35" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H35" s="7"/>
     </row>

</xml_diff>